<commit_message>
Atualiza o acervo com o decreto do CAICA
A planilha da SEPLAN ganhou o Decreto 11.934/2026, que dispoe sobre o
Centro de Atendimento Integrado a Crianca e Adolescente. O acervo passa
de 145 para 146 normas, e os decretos de 5 para 6.

O diff e maior do que a mudanca: o id de cada norma vem da posicao dela
na aba, entao inserir uma no meio renumera as seguintes. O conteudo das
demais nao mudou.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Histórico/HISTÓRICO DE LEIS ORÇAMENTO CRIANÇA E ADOLESCENTE.xlsx
+++ b/Histórico/HISTÓRICO DE LEIS ORÇAMENTO CRIANÇA E ADOLESCENTE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinicius.farias\Desktop\Projeto_OCAD\Histórico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6EE4B69-2B8B-4AFC-B049-E10E65D669BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2EACC8-8B07-457D-AAE3-B20BAD6061AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{22FA6F53-F813-4D91-8754-EDBF1CD8CF6E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{22FA6F53-F813-4D91-8754-EDBF1CD8CF6E}"/>
   </bookViews>
   <sheets>
     <sheet name="Lei Ordinária" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="474" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="476" uniqueCount="371">
   <si>
     <t>Nº da Lei</t>
   </si>
@@ -1242,6 +1242,12 @@
   </si>
   <si>
     <t>SEC. DE ESTADO DE ASSIST. SOCIAL, DA MULHER E DOS DIREITOS HUMANOS - SEAMD/Fundo de Assistência Social - FEAS/Fundo do Direito da Criança e do Adolescente - FDCA/Instituto Sócio Educativo do Acre - ISE/Secretaria Estado de Educação, Cultura e Esportes - SEE</t>
+  </si>
+  <si>
+    <t>DECRETO Nº 11.934, DE 03 DE AGOSTO DE 2026</t>
+  </si>
+  <si>
+    <t>Dispõe sobre o Centro de Atendimento Integrado à Criança e Adolescente - CAICA.</t>
   </si>
 </sst>
 </file>
@@ -2595,8 +2601,12 @@
       <c r="A13" s="25">
         <v>6</v>
       </c>
-      <c r="B13" s="26"/>
-      <c r="C13" s="28"/>
+      <c r="B13" s="26" t="s">
+        <v>369</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>370</v>
+      </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="25">
@@ -2660,9 +2670,10 @@
     <hyperlink ref="B15" r:id="rId3" xr:uid="{55560E2A-6C94-4ED0-8577-7D231457AC28}"/>
     <hyperlink ref="B14" r:id="rId4" xr:uid="{C5882624-4BAE-4DA2-AA08-930B86DCE362}"/>
     <hyperlink ref="B18" r:id="rId5" xr:uid="{6BD0D372-7293-4425-A7E1-B6DE56608B4B}"/>
+    <hyperlink ref="B13" r:id="rId6" xr:uid="{D44A8C6F-A1C1-4622-A50B-4A82E9658983}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Adiciona versao em ingles do site com botao de troca de idioma (PT/EN)
</commit_message>
<xml_diff>
--- a/Histórico/HISTÓRICO DE LEIS ORÇAMENTO CRIANÇA E ADOLESCENTE.xlsx
+++ b/Histórico/HISTÓRICO DE LEIS ORÇAMENTO CRIANÇA E ADOLESCENTE.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vinicius.farias\Desktop\Projeto_OCAD\Histórico\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB2EACC8-8B07-457D-AAE3-B20BAD6061AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECC969F9-C4A3-4216-A729-D2FB3263EED7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{22FA6F53-F813-4D91-8754-EDBF1CD8CF6E}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="5" xr2:uid="{22FA6F53-F813-4D91-8754-EDBF1CD8CF6E}"/>
   </bookViews>
   <sheets>
     <sheet name="Lei Ordinária" sheetId="1" r:id="rId1"/>

</xml_diff>